<commit_message>
Correct draw framing: non-recoverable, not a debt
Clarified with the owner: the draw is NON-RECOVERABLE. Commission offsets the
running balance 100%, but leaving with a balance owes nothing.

The cash mechanics were already modeled correctly, so no formula changed. What
was wrong was the framing: the workbook described the $16,500 as money owed and
flagged it as a liability. It is a balance commission offsets before extra pay
reaches you, and the $36,000/yr draw is a guaranteed floor.

- 41 label and note changes across all 14 sheets removing debt language
- Average loan size default moved to $350,000, giving 1.14 loans/month to hold
  even and an 8-month clear at 2 loans/month
- Values re-baked; 1,687 cells, zero errors

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AxLf3sBNwgqmuMC7wuqj39
</commit_message>
<xml_diff>
--- a/personal-finance/Derek_Roadmap.xlsx
+++ b/personal-finance/Derek_Roadmap.xlsx
@@ -807,7 +807,7 @@
     </comment>
     <comment ref="G7" authorId="0" shapeId="0">
       <text>
-        <t>Confirmed with the owner: 100% of your commission is applied to the outstanding draw. Your example - owe 10,000, commission 2,000, now owe 8,000 - is exactly this column.</t>
+        <t>100% of your commission is applied to the draw balance. Your example - balance 10,000, commission 2,000, balance now 8,000 - is exactly this column. The draw is NON-RECOVERABLE: leave with a balance and you owe nothing.</t>
       </text>
     </comment>
   </commentList>
@@ -1222,11 +1222,11 @@
       </s:c>
       <s:c r="B5" s="7" t="inlineStr">
         <s:is>
-          <s:t>100% of your commission goes to the draw. So until the advance is gone, your take-home is the net draw and nothing else. Closing three loans in a month and closing none feel identical in your bank account. That is not a reason to slow down - it is the reason to speed up, because the only way out is through.</s:t>
-        </s:is>
-      </s:c>
-    </s:row>
-    <s:row r="6" ht="28" customHeight="1">
+          <s:t>The draw is NON-RECOVERABLE: leave tomorrow and you owe nothing, and $36,000/yr is a guaranteed floor. But 100% of commission offsets the running balance, so until it clears your take-home is the net draw. Closing three loans and closing none feel identical in your bank account for now. Not a reason to slow down - the reason to speed up.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="6" ht="39" customHeight="1">
       <s:c r="A6" s="6" t="inlineStr">
         <s:is>
           <s:t>Gross vs net</s:t>
@@ -1234,7 +1234,7 @@
       </s:c>
       <s:c r="B6" s="7" t="inlineStr">
         <s:is>
-          <s:t>The advance grows by the GROSS draw ($1,500 a check), not the $1,231.58 that reaches you. That is why you owe $16,500 after 11 draws, not $13,547. Confirm the $1,500 off a pay stub.</s:t>
+          <s:t>The balance grows by the GROSS draw ($1,500 a check), not the $1,231.58 that reaches you - so it stands at $16,500 after 11 draws, not $13,547. Again: not a debt. Confirm the $1,500 off a pay stub.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -1278,7 +1278,7 @@
       </s:c>
       <s:c r="B10" s="9" t="inlineStr">
         <s:is>
-          <s:t>24 months. Shows exactly when the advance clears and your pay jumps.</s:t>
+          <s:t>24 months. Shows exactly when the balance clears and your pay jumps.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -1510,7 +1510,7 @@
     <s:row r="2" ht="16" customHeight="1">
       <s:c r="A2" s="3" t="inlineStr">
         <s:is>
-          <s:t>Two situations: while the advance is outstanding, and after it clears. Right now you are in the first one.</s:t>
+          <s:t>Two situations: while the draw balance is still being worked through, and after it clears. You are in the first one.</s:t>
         </s:is>
       </s:c>
       <s:c r="B2" s="2" t="n"/>
@@ -1521,7 +1521,7 @@
     <s:row r="4">
       <s:c r="A4" s="95" t="inlineStr">
         <s:is>
-          <s:t>WHILE THE ADVANCE IS OUTSTANDING</s:t>
+          <s:t>WHILE YOU ARE WORKING THROUGH THE DRAW BALANCE</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -1861,7 +1861,7 @@
     <s:row r="6" ht="30" customHeight="1">
       <s:c r="A6" s="8" t="inlineStr">
         <s:is>
-          <s:t>Clear the draw advance</s:t>
+          <s:t>Work through the draw balance</s:t>
         </s:is>
       </s:c>
       <s:c r="B6" s="76">
@@ -1886,7 +1886,7 @@
       </s:c>
       <s:c r="G6" s="20" t="inlineStr">
         <s:is>
-          <s:t>Comes out of commission, not out of your budget. It is the gate on everything else.</s:t>
+          <s:t>Comes out of commission, not your budget. Not a debt - just the gate before extra money reaches you.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -2084,7 +2084,7 @@
       </s:c>
       <s:c r="G14" s="91" t="inlineStr">
         <s:is>
-          <s:t>Negative means these do not all fit yet. That is not a budgeting failure - it is the sheet telling you the answer is more closings, or a later date. Row 7 is excluded from your budget on purpose: the advance is repaid from commission, not from your paycheck.</s:t>
+          <s:t>Negative means these do not all fit yet. That is not a budgeting failure - it is the sheet telling you the answer is more closings, or a later date. Row 7 is excluded from your budget on purpose: the balance is offset by commission, not paid from your paycheck.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -2387,7 +2387,7 @@
     <s:row r="22" ht="30" customHeight="1">
       <s:c r="B22" s="103" t="inlineStr">
         <s:is>
-          <s:t>Commission income normally needs a 2-year history to count as qualifying income. You started 3/31/2026, so your first clean 2-year look is around APRIL 2028. Worse: while the advance is outstanding your W-2 shows the draw only. A lender looks at documented income - and right now that is about $36,000 gross. Verify against current agency guidelines and your AUS findings.</s:t>
+          <s:t>Commission income normally needs a 2-year history to count as qualifying income. You started 3/31/2026, so your first clean 2-year look is around APRIL 2028. Note: while the balance is being worked through your W-2 shows the draw only. A lender looks at documented income - and right now that is about $36,000 gross. Verify against current agency guidelines and your AUS findings.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -3999,7 +3999,7 @@
     <s:row r="2" ht="16" customHeight="1">
       <s:c r="A2" s="3" t="inlineStr">
         <s:is>
-          <s:t>Everything here updates as you log deals. Phase 2 is the wall: until the advance is gone, closing more loans does not raise your pay by one dollar.</s:t>
+          <s:t>Everything here updates as you log deals. Phase 2 is the wall: until the balance is worked through, closing more loans does not raise your pay. But you never OWE it - walk away and it is forgiven.</s:t>
         </s:is>
       </s:c>
       <s:c r="B2" s="2" t="n"/>
@@ -4016,8 +4016,8 @@
         </s:is>
       </s:c>
       <s:c r="C4" s="13" t="str">
-        <s:f>IF(Inputs!$C$17&gt;0,"PHASE 2 - digging out from under the advance","PHASE 3+ - the advance is clear")</s:f>
-        <s:v>PHASE 2 - digging out from under the advance</s:v>
+        <s:f>IF(Inputs!$C$17&gt;0,"PHASE 2 - working through the draw balance","PHASE 3+ - balance clear, commission is yours")</s:f>
+        <s:v>PHASE 2 - working through the draw balance</s:v>
       </s:c>
       <s:c r="D4" s="14" t="n"/>
       <s:c r="E4" s="14" t="n"/>
@@ -4060,12 +4060,12 @@
     <s:row r="6" ht="44" customHeight="1">
       <s:c r="B6" s="8" t="inlineStr">
         <s:is>
-          <s:t>1. Stop the advance growing</s:t>
+          <s:t>1. Stop the balance growing</s:t>
         </s:is>
       </s:c>
       <s:c r="C6" s="17">
         <s:f>Inputs!$C$24</s:f>
-        <s:v>1.3333333333333333</s:v>
+        <s:v>1.1428571428571428</s:v>
       </s:c>
       <s:c r="D6" s="17">
         <s:f>Inputs!$C$20</s:f>
@@ -4081,14 +4081,14 @@
       </s:c>
       <s:c r="G6" s="20" t="inlineStr">
         <s:is>
-          <s:t>At 1 loan/month the advance still GROWS by $750. You need 1.33 loans a month at $300k just to hold even. This is the first real milestone and it is lower than it feels.</s:t>
+          <s:t>At 1 loan/month the balance still GROWS by $750. You need 1.33 loans/mo at $300k to hold even - only 1.14 at $350k. First real milestone, and lower than it feels.</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="7" ht="44" customHeight="1">
       <s:c r="B7" s="21" t="inlineStr">
         <s:is>
-          <s:t>2. Clear the advance</s:t>
+          <s:t>2. Work through the balance</s:t>
         </s:is>
       </s:c>
       <s:c r="C7" s="22">
@@ -4109,7 +4109,7 @@
       </s:c>
       <s:c r="G7" s="24" t="inlineStr">
         <s:is>
-          <s:t>100% of commission goes here. Until it hits zero your take-home is the net draw and nothing more. The Draw Payback tab dates this precisely.</s:t>
+          <s:t>100% of commission goes here. Until it hits zero your take-home is the net draw. NOT a debt - leave tomorrow and you owe nothing. The Draw Payback tab dates it precisely.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4213,12 +4213,12 @@
     <s:row r="13">
       <s:c r="B13" s="8" t="inlineStr">
         <s:is>
-          <s:t>Advance clears</s:t>
+          <s:t>Balance clears</s:t>
         </s:is>
       </s:c>
       <s:c r="C13" s="13" t="str">
         <s:f>'Draw Payback'!D4</s:f>
-        <s:v>11 months</s:v>
+        <s:v>8 months</s:v>
       </s:c>
       <s:c r="D13" s="15" t="n"/>
       <s:c r="G13" s="20" t="inlineStr">
@@ -4235,7 +4235,7 @@
       </s:c>
       <s:c r="C14" s="13">
         <s:f>'Draw Payback'!H4</s:f>
-        <s:v>46599.0</s:v>
+        <s:v>46507.0</s:v>
       </s:c>
       <s:c r="D14" s="15" t="n"/>
       <s:c r="G14" s="24" t="inlineStr">
@@ -4252,7 +4252,7 @@
       </s:c>
       <s:c r="C15" s="26">
         <s:f>Inputs!$C$24</s:f>
-        <s:v>1.3333333333333333</s:v>
+        <s:v>1.1428571428571428</s:v>
       </s:c>
       <s:c r="D15" s="15" t="n"/>
       <s:c r="G15" s="20" t="inlineStr">
@@ -4367,8 +4367,8 @@
     </s:row>
     <s:row r="2" ht="16" customHeight="1">
       <s:c r="A2" s="3" t="str">
-        <s:f>"Model date "&amp;TEXT(Inputs!$C$59,"mmm d, yyyy")&amp;"   |   Draw is RECOVERABLE, commission 100% recaptured   |   W-2, taxes withheld   |   Planning "&amp;TEXT(Inputs!$C$20,"0.0")&amp;" loans/month"</s:f>
-        <s:v>Model date Sep 1, 2026   |   Draw is RECOVERABLE, commission 100% recaptured   |   W-2, taxes withheld   |   Planning 2.0 loans/month</s:v>
+        <s:f>"Model date "&amp;TEXT(Inputs!$C$59,"mmm d, yyyy")&amp;"   |   Draw NON-RECOVERABLE (forgiven if you leave), commission offsets it 100%   |   W-2, taxes withheld   |   Planning "&amp;TEXT(Inputs!$C$20,"0.0")&amp;" loans/month"</s:f>
+        <s:v>Model date Sep 1, 2026   |   Draw NON-RECOVERABLE (forgiven if you leave), commission offsets it 100%   |   W-2, taxes withheld   |   Planning 2.0 loans/month</s:v>
       </s:c>
       <s:c r="B2" s="2" t="n"/>
       <s:c r="C2" s="2" t="n"/>
@@ -4389,7 +4389,7 @@
     <s:row r="5">
       <s:c r="B5" s="28" t="inlineStr">
         <s:is>
-          <s:t>You owe on the draw</s:t>
+          <s:t>Draw balance to work through</s:t>
         </s:is>
       </s:c>
       <s:c r="C5" s="29">
@@ -4403,7 +4403,7 @@
       </s:c>
       <s:c r="F5" s="30">
         <s:f>Inputs!$C$24</s:f>
-        <s:v>1.3333333333333333</s:v>
+        <s:v>1.1428571428571428</s:v>
       </s:c>
       <s:c r="H5" s="28" t="inlineStr">
         <s:is>
@@ -4447,21 +4447,21 @@
     <s:row r="7">
       <s:c r="B7" s="28" t="inlineStr">
         <s:is>
-          <s:t>Advance clears in</s:t>
+          <s:t>Balance clears in</s:t>
         </s:is>
       </s:c>
       <s:c r="C7" s="13" t="str">
         <s:f>'Draw Payback'!D4</s:f>
-        <s:v>11 months</s:v>
+        <s:v>8 months</s:v>
       </s:c>
       <s:c r="E7" s="28" t="inlineStr">
         <s:is>
-          <s:t>Advance moves per month</s:t>
+          <s:t>Balance moves per month</s:t>
         </s:is>
       </s:c>
       <s:c r="F7" s="32">
         <s:f>Inputs!$C$22</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H7" s="28" t="inlineStr">
         <s:is>
@@ -4541,7 +4541,7 @@
     <s:row r="12">
       <s:c r="B12" s="34" t="inlineStr">
         <s:is>
-          <s:t>1.  Confirm the gross draw is $1,500 off a pay stub. Every number here scales off it.</s:t>
+          <s:t>1.  Confirm the gross draw is $1,500 off a pay stub, AND whether the balance resets on January 1. Most non-recoverable draws do.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4656,7 +4656,7 @@
       </s:c>
       <s:c r="E5" s="38" t="inlineStr">
         <s:is>
-          <s:t>You said 'I think it's 1500'. CONFIRM off a pay stub - this is the number the advance grows by, so it drives everything.</s:t>
+          <s:t>You said 'I think it's 1500'. CONFIRM off a pay stub - this is the number the balance grows by, so it drives everything.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4734,7 +4734,7 @@
       </s:c>
       <s:c r="E9" s="38" t="inlineStr">
         <s:is>
-          <s:t>The advance grows by this every month.</s:t>
+          <s:t>The balance grows by this every month.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4755,7 +4755,7 @@
       </s:c>
       <s:c r="E10" s="38" t="inlineStr">
         <s:is>
-          <s:t>This is your entire income until the advance is cleared, no matter how much you close.</s:t>
+          <s:t>This is your entire income until the balance is worked through, no matter how much you close.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4807,14 +4807,14 @@
       <s:c r="D13" s="37" t="inlineStr"/>
       <s:c r="E13" s="38" t="inlineStr">
         <s:is>
-          <s:t>Commission is usually withheld at the 22% federal supplemental rate plus state. Only matters once the advance clears.</s:t>
+          <s:t>Commission is usually withheld at the 22% federal supplemental rate plus state. Only matters once the balance is worked through.</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="14" ht="19" customHeight="1">
       <s:c r="A14" s="4" t="inlineStr">
         <s:is>
-          <s:t xml:space="preserve">  2.  THE ADVANCE  —  confirmed: 100% of your commission goes to the draw</s:t>
+          <s:t xml:space="preserve">  2.  THE DRAW BALANCE  —  NON-RECOVERABLE. Commission offsets it, but you never owe it.</s:t>
         </s:is>
       </s:c>
       <s:c r="B14" s="5" t="n"/>
@@ -4825,7 +4825,7 @@
     <s:row r="15" ht="28" customHeight="1">
       <s:c r="B15" s="12" t="inlineStr">
         <s:is>
-          <s:t>Advance from draws taken</s:t>
+          <s:t>Draw paid to you so far</s:t>
         </s:is>
       </s:c>
       <s:c r="C15" s="44">
@@ -4839,7 +4839,7 @@
       </s:c>
       <s:c r="E15" s="38" t="inlineStr">
         <s:is>
-          <s:t>11 x $1,500 GROSS. Note this is $2,952.62 higher than a net-based figure - the company advanced the gross.</s:t>
+          <s:t>11 x $1,500 GROSS. This is NOT a debt. It is the amount your commissions offset against before extra money reaches you.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4864,10 +4864,10 @@
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="17">
+    <s:row r="17" ht="28" customHeight="1">
       <s:c r="B17" s="12" t="inlineStr">
         <s:is>
-          <s:t>YOU CURRENTLY OWE</s:t>
+          <s:t>BALANCE STILL TO WORK THROUGH</s:t>
         </s:is>
       </s:c>
       <s:c r="C17" s="44">
@@ -4881,7 +4881,7 @@
       </s:c>
       <s:c r="E17" s="38" t="inlineStr">
         <s:is>
-          <s:t>Log deals and watch this fall.</s:t>
+          <s:t>NOT money you owe. If you left tomorrow you would owe nothing - it is simply what commission offsets before you get paid on top. Log deals and watch it fall.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4903,7 +4903,7 @@
         </s:is>
       </s:c>
       <s:c r="C19" s="45" t="n">
-        <s:v>300000</s:v>
+        <s:v>350000</s:v>
       </s:c>
       <s:c r="D19" s="37" t="inlineStr">
         <s:is>
@@ -4912,11 +4912,11 @@
       </s:c>
       <s:c r="E19" s="38" t="inlineStr">
         <s:is>
-          <s:t>Set from your real pipeline.</s:t>
-        </s:is>
-      </s:c>
-    </s:row>
-    <s:row r="20">
+          <s:t>Your working number. At 75 bps a $350k loan pays you $2,625.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="20" ht="28" customHeight="1">
       <s:c r="B20" s="35" t="inlineStr">
         <s:is>
           <s:t>Loans per month you PLAN to close</s:t>
@@ -4932,7 +4932,7 @@
       </s:c>
       <s:c r="E20" s="38" t="inlineStr">
         <s:is>
-          <s:t>Change this and the whole roadmap re-times.</s:t>
+          <s:t>You closed 2 in September (9/9 and 9/18) after five months of none - that is the pipeline turning on. Change this and the whole roadmap re-times.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -4944,7 +4944,7 @@
       </s:c>
       <s:c r="C21" s="41">
         <s:f>C20*C19*C12</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="D21" s="37" t="inlineStr">
         <s:is>
@@ -4956,12 +4956,12 @@
     <s:row r="22">
       <s:c r="B22" s="12" t="inlineStr">
         <s:is>
-          <s:t xml:space="preserve">  = pays down the advance by</s:t>
+          <s:t xml:space="preserve">  = works the balance down by</s:t>
         </s:is>
       </s:c>
       <s:c r="C22" s="41">
         <s:f>C21-C9</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="D22" s="37" t="inlineStr">
         <s:is>
@@ -4974,7 +4974,7 @@
         </s:is>
       </s:c>
     </s:row>
-    <s:row r="23">
+    <s:row r="23" ht="28" customHeight="1">
       <s:c r="B23" s="12" t="inlineStr">
         <s:is>
           <s:t>BREAK-EVEN: commission needed just to STOP the balance growing</s:t>
@@ -4991,11 +4991,11 @@
       </s:c>
       <s:c r="E23" s="38" t="inlineStr">
         <s:is>
-          <s:t>Below this the advance gets BIGGER every month even though you are closing loans.</s:t>
-        </s:is>
-      </s:c>
-    </s:row>
-    <s:row r="24" ht="28" customHeight="1">
+          <s:t>Below this the balance gets BIGGER every month even though you are closing loans. Not a debt - just a longer wait before extra money reaches you.</s:t>
+        </s:is>
+      </s:c>
+    </s:row>
+    <s:row r="24">
       <s:c r="B24" s="12" t="inlineStr">
         <s:is>
           <s:t xml:space="preserve">  = loans per month to stop digging</s:t>
@@ -5003,7 +5003,7 @@
       </s:c>
       <s:c r="C24" s="47">
         <s:f>C23/C12/C19</s:f>
-        <s:v>1.3333333333333333</s:v>
+        <s:v>1.1428571428571428</s:v>
       </s:c>
       <s:c r="D24" s="37" t="inlineStr">
         <s:is>
@@ -5012,19 +5012,19 @@
       </s:c>
       <s:c r="E24" s="38" t="inlineStr">
         <s:is>
-          <s:t>THE number that matters most right now. At 1 loan/month the advance still grows by $750 every month.</s:t>
+          <s:t>THE number that matters most. At 1 loan/month the balance still grows by $750 a month.</s:t>
         </s:is>
       </s:c>
     </s:row>
     <s:row r="25">
       <s:c r="B25" s="12" t="inlineStr">
         <s:is>
-          <s:t>Months to clear the advance at your planned pace</s:t>
+          <s:t>Months to work through the balance at your planned pace</s:t>
         </s:is>
       </s:c>
       <s:c r="C25" s="48">
         <s:f>IF(C22&lt;=0,"never at this pace",ROUNDUP(C17/C22,0))</s:f>
-        <s:v>11.0</s:v>
+        <s:v>8.0</s:v>
       </s:c>
       <s:c r="D25" s="37" t="inlineStr">
         <s:is>
@@ -5803,7 +5803,7 @@
     <s:row r="5">
       <s:c r="A5" s="12" t="inlineStr">
         <s:is>
-          <s:t>Still owed on the draw</s:t>
+          <s:t>Draw balance to work through</s:t>
         </s:is>
       </s:c>
       <s:c r="C5" s="29">
@@ -10401,7 +10401,7 @@
     <s:row r="4">
       <s:c r="A4" s="12" t="inlineStr">
         <s:is>
-          <s:t>Advance today</s:t>
+          <s:t>Balance today</s:t>
         </s:is>
       </s:c>
       <s:c r="B4" s="29">
@@ -10415,7 +10415,7 @@
       </s:c>
       <s:c r="D4" s="13" t="str">
         <s:f>IFERROR(MATCH(0,F9:F32,0)&amp;" months","not within 24 mo")</s:f>
-        <s:v>11 months</s:v>
+        <s:v>8 months</s:v>
       </s:c>
       <s:c r="E4" s="12" t="inlineStr">
         <s:is>
@@ -10424,13 +10424,13 @@
       </s:c>
       <s:c r="H4" s="75">
         <s:f>IFERROR(INDEX(A9:A32,MATCH(0,F9:F32,0)),"not within 24 months")</s:f>
-        <s:v>46599.0</s:v>
+        <s:v>46507.0</s:v>
       </s:c>
     </s:row>
     <s:row r="5">
       <s:c r="A5" s="53" t="str">
         <s:f>"At your planned pace of "&amp;TEXT(Inputs!$C$20,"0.0")&amp;" loans/month you earn "&amp;TEXT(Inputs!$C$21,"$#,##0")&amp;" while the draw adds "&amp;TEXT(Inputs!$C$9,"$#,##0")&amp;" - so the balance moves "&amp;TEXT(Inputs!$C$22,"$#,##0")&amp;" a month."</s:f>
-        <s:v>At your planned pace of 2.0 loans/month you earn $4,500 while the draw adds $3,000 - so the balance moves $1,500 a month.</s:v>
+        <s:v>At your planned pace of 2.0 loans/month you earn $5,250 while the draw adds $3,000 - so the balance moves $2,250 a month.</s:v>
       </s:c>
     </s:row>
     <s:row r="8" ht="30" customHeight="1">
@@ -10442,7 +10442,7 @@
       <s:c r="B8" s="16" t="inlineStr">
         <s:is>
           <s:t>Opening
-advance</s:t>
+balance</s:t>
         </s:is>
       </s:c>
       <s:c r="C8" s="16" t="inlineStr">
@@ -10460,13 +10460,13 @@
       <s:c r="E8" s="16" t="inlineStr">
         <s:is>
           <s:t>Applied to
-advance</s:t>
+balance</s:t>
         </s:is>
       </s:c>
       <s:c r="F8" s="16" t="inlineStr">
         <s:is>
           <s:t>Closing
-advance</s:t>
+balance</s:t>
         </s:is>
       </s:c>
       <s:c r="G8" s="16" t="inlineStr">
@@ -10513,15 +10513,15 @@
       </s:c>
       <s:c r="D9" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A9,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A9,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E9" s="76">
         <s:f>MIN(B9+C9,D9)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F9" s="77">
         <s:f>MAX(0,B9+C9-D9)</s:f>
-        <s:v>15000.0</s:v>
+        <s:v>14250.0</s:v>
       </s:c>
       <s:c r="G9" s="76">
         <s:f>MAX(0,D9-(B9+C9))</s:f>
@@ -10540,8 +10540,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K9" s="78" t="str">
-        <s:f>IF(F9&gt;B9,"Advance still growing",IF(F9&gt;0,"Paying it down",IF(G9&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F9&gt;B9,"Balance still growing",IF(F9&gt;0,"Working it down",IF(G9&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="10">
@@ -10551,7 +10551,7 @@
       </s:c>
       <s:c r="B10" s="79">
         <s:f>F9</s:f>
-        <s:v>15000.0</s:v>
+        <s:v>14250.0</s:v>
       </s:c>
       <s:c r="C10" s="73">
         <s:f>Inputs!$C$9</s:f>
@@ -10559,15 +10559,15 @@
       </s:c>
       <s:c r="D10" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A10,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A10,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E10" s="79">
         <s:f>MIN(B10+C10,D10)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F10" s="80">
         <s:f>MAX(0,B10+C10-D10)</s:f>
-        <s:v>13500.0</s:v>
+        <s:v>12000.0</s:v>
       </s:c>
       <s:c r="G10" s="79">
         <s:f>MAX(0,D10-(B10+C10))</s:f>
@@ -10586,8 +10586,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K10" s="81" t="str">
-        <s:f>IF(F10&gt;B10,"Advance still growing",IF(F10&gt;0,"Paying it down",IF(G10&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F10&gt;B10,"Balance still growing",IF(F10&gt;0,"Working it down",IF(G10&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="11">
@@ -10597,7 +10597,7 @@
       </s:c>
       <s:c r="B11" s="76">
         <s:f>F10</s:f>
-        <s:v>13500.0</s:v>
+        <s:v>12000.0</s:v>
       </s:c>
       <s:c r="C11" s="67">
         <s:f>Inputs!$C$9</s:f>
@@ -10605,15 +10605,15 @@
       </s:c>
       <s:c r="D11" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A11,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A11,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E11" s="76">
         <s:f>MIN(B11+C11,D11)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F11" s="77">
         <s:f>MAX(0,B11+C11-D11)</s:f>
-        <s:v>12000.0</s:v>
+        <s:v>9750.0</s:v>
       </s:c>
       <s:c r="G11" s="76">
         <s:f>MAX(0,D11-(B11+C11))</s:f>
@@ -10632,8 +10632,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K11" s="78" t="str">
-        <s:f>IF(F11&gt;B11,"Advance still growing",IF(F11&gt;0,"Paying it down",IF(G11&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F11&gt;B11,"Balance still growing",IF(F11&gt;0,"Working it down",IF(G11&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="12">
@@ -10643,7 +10643,7 @@
       </s:c>
       <s:c r="B12" s="79">
         <s:f>F11</s:f>
-        <s:v>12000.0</s:v>
+        <s:v>9750.0</s:v>
       </s:c>
       <s:c r="C12" s="73">
         <s:f>Inputs!$C$9</s:f>
@@ -10651,15 +10651,15 @@
       </s:c>
       <s:c r="D12" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A12,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A12,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E12" s="79">
         <s:f>MIN(B12+C12,D12)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F12" s="80">
         <s:f>MAX(0,B12+C12-D12)</s:f>
-        <s:v>10500.0</s:v>
+        <s:v>7500.0</s:v>
       </s:c>
       <s:c r="G12" s="79">
         <s:f>MAX(0,D12-(B12+C12))</s:f>
@@ -10678,8 +10678,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K12" s="81" t="str">
-        <s:f>IF(F12&gt;B12,"Advance still growing",IF(F12&gt;0,"Paying it down",IF(G12&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F12&gt;B12,"Balance still growing",IF(F12&gt;0,"Working it down",IF(G12&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="13">
@@ -10689,7 +10689,7 @@
       </s:c>
       <s:c r="B13" s="76">
         <s:f>F12</s:f>
-        <s:v>10500.0</s:v>
+        <s:v>7500.0</s:v>
       </s:c>
       <s:c r="C13" s="67">
         <s:f>Inputs!$C$9</s:f>
@@ -10697,15 +10697,15 @@
       </s:c>
       <s:c r="D13" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A13,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A13,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E13" s="76">
         <s:f>MIN(B13+C13,D13)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F13" s="77">
         <s:f>MAX(0,B13+C13-D13)</s:f>
-        <s:v>9000.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="G13" s="76">
         <s:f>MAX(0,D13-(B13+C13))</s:f>
@@ -10724,8 +10724,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K13" s="78" t="str">
-        <s:f>IF(F13&gt;B13,"Advance still growing",IF(F13&gt;0,"Paying it down",IF(G13&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F13&gt;B13,"Balance still growing",IF(F13&gt;0,"Working it down",IF(G13&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="14">
@@ -10735,7 +10735,7 @@
       </s:c>
       <s:c r="B14" s="79">
         <s:f>F13</s:f>
-        <s:v>9000.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="C14" s="73">
         <s:f>Inputs!$C$9</s:f>
@@ -10743,15 +10743,15 @@
       </s:c>
       <s:c r="D14" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A14,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A14,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E14" s="79">
         <s:f>MIN(B14+C14,D14)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F14" s="80">
         <s:f>MAX(0,B14+C14-D14)</s:f>
-        <s:v>7500.0</s:v>
+        <s:v>3000.0</s:v>
       </s:c>
       <s:c r="G14" s="79">
         <s:f>MAX(0,D14-(B14+C14))</s:f>
@@ -10770,8 +10770,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K14" s="81" t="str">
-        <s:f>IF(F14&gt;B14,"Advance still growing",IF(F14&gt;0,"Paying it down",IF(G14&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F14&gt;B14,"Balance still growing",IF(F14&gt;0,"Working it down",IF(G14&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="15">
@@ -10781,7 +10781,7 @@
       </s:c>
       <s:c r="B15" s="76">
         <s:f>F14</s:f>
-        <s:v>7500.0</s:v>
+        <s:v>3000.0</s:v>
       </s:c>
       <s:c r="C15" s="67">
         <s:f>Inputs!$C$9</s:f>
@@ -10789,15 +10789,15 @@
       </s:c>
       <s:c r="D15" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A15,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A15,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E15" s="76">
         <s:f>MIN(B15+C15,D15)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="F15" s="77">
         <s:f>MAX(0,B15+C15-D15)</s:f>
-        <s:v>6000.0</s:v>
+        <s:v>750.0</s:v>
       </s:c>
       <s:c r="G15" s="76">
         <s:f>MAX(0,D15-(B15+C15))</s:f>
@@ -10816,8 +10816,8 @@
         <s:v>2463.16</s:v>
       </s:c>
       <s:c r="K15" s="78" t="str">
-        <s:f>IF(F15&gt;B15,"Advance still growing",IF(F15&gt;0,"Paying it down",IF(G15&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F15&gt;B15,"Balance still growing",IF(F15&gt;0,"Working it down",IF(G15&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>Working it down</s:v>
       </s:c>
     </s:row>
     <s:row r="16">
@@ -10827,7 +10827,7 @@
       </s:c>
       <s:c r="B16" s="79">
         <s:f>F15</s:f>
-        <s:v>6000.0</s:v>
+        <s:v>750.0</s:v>
       </s:c>
       <s:c r="C16" s="73">
         <s:f>Inputs!$C$9</s:f>
@@ -10835,23 +10835,23 @@
       </s:c>
       <s:c r="D16" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A16,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A16,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E16" s="79">
         <s:f>MIN(B16+C16,D16)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>3750.0</s:v>
       </s:c>
       <s:c r="F16" s="80">
         <s:f>MAX(0,B16+C16-D16)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="G16" s="79">
         <s:f>MAX(0,D16-(B16+C16))</s:f>
-        <s:v>0.0</s:v>
+        <s:v>1500.0</s:v>
       </s:c>
       <s:c r="H16" s="79">
         <s:f>G16*Inputs!$C$13</s:f>
-        <s:v>0.0</s:v>
+        <s:v>330.0</s:v>
       </s:c>
       <s:c r="I16" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -10859,11 +10859,11 @@
       </s:c>
       <s:c r="J16" s="66">
         <s:f>I16+G16-H16</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>3633.16</s:v>
       </s:c>
       <s:c r="K16" s="81" t="str">
-        <s:f>IF(F16&gt;B16,"Advance still growing",IF(F16&gt;0,"Paying it down",IF(G16&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F16&gt;B16,"Balance still growing",IF(F16&gt;0,"Working it down",IF(G16&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
     <s:row r="17">
@@ -10873,7 +10873,7 @@
       </s:c>
       <s:c r="B17" s="76">
         <s:f>F16</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="C17" s="67">
         <s:f>Inputs!$C$9</s:f>
@@ -10881,23 +10881,23 @@
       </s:c>
       <s:c r="D17" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A17,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A17,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E17" s="76">
         <s:f>MIN(B17+C17,D17)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>3000.0</s:v>
       </s:c>
       <s:c r="F17" s="77">
         <s:f>MAX(0,B17+C17-D17)</s:f>
-        <s:v>3000.0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="G17" s="76">
         <s:f>MAX(0,D17-(B17+C17))</s:f>
-        <s:v>0.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H17" s="76">
         <s:f>G17*Inputs!$C$13</s:f>
-        <s:v>0.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I17" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -10905,11 +10905,11 @@
       </s:c>
       <s:c r="J17" s="66">
         <s:f>I17+G17-H17</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K17" s="78" t="str">
-        <s:f>IF(F17&gt;B17,"Advance still growing",IF(F17&gt;0,"Paying it down",IF(G17&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F17&gt;B17,"Balance still growing",IF(F17&gt;0,"Working it down",IF(G17&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
     <s:row r="18">
@@ -10919,7 +10919,7 @@
       </s:c>
       <s:c r="B18" s="79">
         <s:f>F17</s:f>
-        <s:v>3000.0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="C18" s="73">
         <s:f>Inputs!$C$9</s:f>
@@ -10927,23 +10927,23 @@
       </s:c>
       <s:c r="D18" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A18,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A18,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E18" s="79">
         <s:f>MIN(B18+C18,D18)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>3000.0</s:v>
       </s:c>
       <s:c r="F18" s="80">
         <s:f>MAX(0,B18+C18-D18)</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="G18" s="79">
         <s:f>MAX(0,D18-(B18+C18))</s:f>
-        <s:v>0.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H18" s="79">
         <s:f>G18*Inputs!$C$13</s:f>
-        <s:v>0.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I18" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -10951,11 +10951,11 @@
       </s:c>
       <s:c r="J18" s="66">
         <s:f>I18+G18-H18</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K18" s="81" t="str">
-        <s:f>IF(F18&gt;B18,"Advance still growing",IF(F18&gt;0,"Paying it down",IF(G18&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Paying it down</s:v>
+        <s:f>IF(F18&gt;B18,"Balance still growing",IF(F18&gt;0,"Working it down",IF(G18&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
     <s:row r="19">
@@ -10965,7 +10965,7 @@
       </s:c>
       <s:c r="B19" s="76">
         <s:f>F18</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>0.0</s:v>
       </s:c>
       <s:c r="C19" s="67">
         <s:f>Inputs!$C$9</s:f>
@@ -10973,11 +10973,11 @@
       </s:c>
       <s:c r="D19" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A19,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A19,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E19" s="76">
         <s:f>MIN(B19+C19,D19)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>3000.0</s:v>
       </s:c>
       <s:c r="F19" s="77">
         <s:f>MAX(0,B19+C19-D19)</s:f>
@@ -10985,11 +10985,11 @@
       </s:c>
       <s:c r="G19" s="76">
         <s:f>MAX(0,D19-(B19+C19))</s:f>
-        <s:v>0.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H19" s="76">
         <s:f>G19*Inputs!$C$13</s:f>
-        <s:v>0.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I19" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -10997,11 +10997,11 @@
       </s:c>
       <s:c r="J19" s="66">
         <s:f>I19+G19-H19</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K19" s="78" t="str">
-        <s:f>IF(F19&gt;B19,"Advance still growing",IF(F19&gt;0,"Paying it down",IF(G19&gt;0,"CLEARED - real income now","Cleared")))</s:f>
-        <s:v>Cleared</s:v>
+        <s:f>IF(F19&gt;B19,"Balance still growing",IF(F19&gt;0,"Working it down",IF(G19&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
     <s:row r="20">
@@ -11019,7 +11019,7 @@
       </s:c>
       <s:c r="D20" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A20,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A20,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E20" s="79">
         <s:f>MIN(B20+C20,D20)</s:f>
@@ -11031,11 +11031,11 @@
       </s:c>
       <s:c r="G20" s="79">
         <s:f>MAX(0,D20-(B20+C20))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H20" s="79">
         <s:f>G20*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I20" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11043,10 +11043,10 @@
       </s:c>
       <s:c r="J20" s="66">
         <s:f>I20+G20-H20</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K20" s="81" t="str">
-        <s:f>IF(F20&gt;B20,"Advance still growing",IF(F20&gt;0,"Paying it down",IF(G20&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F20&gt;B20,"Balance still growing",IF(F20&gt;0,"Working it down",IF(G20&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11065,7 +11065,7 @@
       </s:c>
       <s:c r="D21" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A21,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A21,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E21" s="76">
         <s:f>MIN(B21+C21,D21)</s:f>
@@ -11077,11 +11077,11 @@
       </s:c>
       <s:c r="G21" s="76">
         <s:f>MAX(0,D21-(B21+C21))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H21" s="76">
         <s:f>G21*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I21" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -11089,10 +11089,10 @@
       </s:c>
       <s:c r="J21" s="66">
         <s:f>I21+G21-H21</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K21" s="78" t="str">
-        <s:f>IF(F21&gt;B21,"Advance still growing",IF(F21&gt;0,"Paying it down",IF(G21&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F21&gt;B21,"Balance still growing",IF(F21&gt;0,"Working it down",IF(G21&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11111,7 +11111,7 @@
       </s:c>
       <s:c r="D22" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A22,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A22,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E22" s="79">
         <s:f>MIN(B22+C22,D22)</s:f>
@@ -11123,11 +11123,11 @@
       </s:c>
       <s:c r="G22" s="79">
         <s:f>MAX(0,D22-(B22+C22))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H22" s="79">
         <s:f>G22*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I22" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11135,10 +11135,10 @@
       </s:c>
       <s:c r="J22" s="66">
         <s:f>I22+G22-H22</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K22" s="81" t="str">
-        <s:f>IF(F22&gt;B22,"Advance still growing",IF(F22&gt;0,"Paying it down",IF(G22&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F22&gt;B22,"Balance still growing",IF(F22&gt;0,"Working it down",IF(G22&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11157,7 +11157,7 @@
       </s:c>
       <s:c r="D23" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A23,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A23,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E23" s="76">
         <s:f>MIN(B23+C23,D23)</s:f>
@@ -11169,11 +11169,11 @@
       </s:c>
       <s:c r="G23" s="76">
         <s:f>MAX(0,D23-(B23+C23))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H23" s="76">
         <s:f>G23*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I23" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -11181,10 +11181,10 @@
       </s:c>
       <s:c r="J23" s="66">
         <s:f>I23+G23-H23</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K23" s="78" t="str">
-        <s:f>IF(F23&gt;B23,"Advance still growing",IF(F23&gt;0,"Paying it down",IF(G23&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F23&gt;B23,"Balance still growing",IF(F23&gt;0,"Working it down",IF(G23&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11203,7 +11203,7 @@
       </s:c>
       <s:c r="D24" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A24,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A24,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E24" s="79">
         <s:f>MIN(B24+C24,D24)</s:f>
@@ -11215,11 +11215,11 @@
       </s:c>
       <s:c r="G24" s="79">
         <s:f>MAX(0,D24-(B24+C24))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H24" s="79">
         <s:f>G24*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I24" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11227,10 +11227,10 @@
       </s:c>
       <s:c r="J24" s="66">
         <s:f>I24+G24-H24</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K24" s="81" t="str">
-        <s:f>IF(F24&gt;B24,"Advance still growing",IF(F24&gt;0,"Paying it down",IF(G24&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F24&gt;B24,"Balance still growing",IF(F24&gt;0,"Working it down",IF(G24&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11249,7 +11249,7 @@
       </s:c>
       <s:c r="D25" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A25,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A25,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E25" s="76">
         <s:f>MIN(B25+C25,D25)</s:f>
@@ -11261,11 +11261,11 @@
       </s:c>
       <s:c r="G25" s="76">
         <s:f>MAX(0,D25-(B25+C25))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H25" s="76">
         <s:f>G25*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I25" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -11273,10 +11273,10 @@
       </s:c>
       <s:c r="J25" s="66">
         <s:f>I25+G25-H25</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K25" s="78" t="str">
-        <s:f>IF(F25&gt;B25,"Advance still growing",IF(F25&gt;0,"Paying it down",IF(G25&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F25&gt;B25,"Balance still growing",IF(F25&gt;0,"Working it down",IF(G25&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11295,7 +11295,7 @@
       </s:c>
       <s:c r="D26" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A26,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A26,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E26" s="79">
         <s:f>MIN(B26+C26,D26)</s:f>
@@ -11307,11 +11307,11 @@
       </s:c>
       <s:c r="G26" s="79">
         <s:f>MAX(0,D26-(B26+C26))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H26" s="79">
         <s:f>G26*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I26" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11319,10 +11319,10 @@
       </s:c>
       <s:c r="J26" s="66">
         <s:f>I26+G26-H26</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K26" s="81" t="str">
-        <s:f>IF(F26&gt;B26,"Advance still growing",IF(F26&gt;0,"Paying it down",IF(G26&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F26&gt;B26,"Balance still growing",IF(F26&gt;0,"Working it down",IF(G26&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11341,7 +11341,7 @@
       </s:c>
       <s:c r="D27" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A27,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A27,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E27" s="76">
         <s:f>MIN(B27+C27,D27)</s:f>
@@ -11353,11 +11353,11 @@
       </s:c>
       <s:c r="G27" s="76">
         <s:f>MAX(0,D27-(B27+C27))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H27" s="76">
         <s:f>G27*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I27" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -11365,10 +11365,10 @@
       </s:c>
       <s:c r="J27" s="66">
         <s:f>I27+G27-H27</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K27" s="78" t="str">
-        <s:f>IF(F27&gt;B27,"Advance still growing",IF(F27&gt;0,"Paying it down",IF(G27&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F27&gt;B27,"Balance still growing",IF(F27&gt;0,"Working it down",IF(G27&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11387,7 +11387,7 @@
       </s:c>
       <s:c r="D28" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A28,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A28,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E28" s="79">
         <s:f>MIN(B28+C28,D28)</s:f>
@@ -11399,11 +11399,11 @@
       </s:c>
       <s:c r="G28" s="79">
         <s:f>MAX(0,D28-(B28+C28))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H28" s="79">
         <s:f>G28*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I28" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11411,10 +11411,10 @@
       </s:c>
       <s:c r="J28" s="66">
         <s:f>I28+G28-H28</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K28" s="81" t="str">
-        <s:f>IF(F28&gt;B28,"Advance still growing",IF(F28&gt;0,"Paying it down",IF(G28&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F28&gt;B28,"Balance still growing",IF(F28&gt;0,"Working it down",IF(G28&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11433,7 +11433,7 @@
       </s:c>
       <s:c r="D29" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A29,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A29,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E29" s="76">
         <s:f>MIN(B29+C29,D29)</s:f>
@@ -11445,11 +11445,11 @@
       </s:c>
       <s:c r="G29" s="76">
         <s:f>MAX(0,D29-(B29+C29))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H29" s="76">
         <s:f>G29*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I29" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -11457,10 +11457,10 @@
       </s:c>
       <s:c r="J29" s="66">
         <s:f>I29+G29-H29</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K29" s="78" t="str">
-        <s:f>IF(F29&gt;B29,"Advance still growing",IF(F29&gt;0,"Paying it down",IF(G29&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F29&gt;B29,"Balance still growing",IF(F29&gt;0,"Working it down",IF(G29&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11479,7 +11479,7 @@
       </s:c>
       <s:c r="D30" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A30,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A30,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E30" s="79">
         <s:f>MIN(B30+C30,D30)</s:f>
@@ -11491,11 +11491,11 @@
       </s:c>
       <s:c r="G30" s="79">
         <s:f>MAX(0,D30-(B30+C30))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H30" s="79">
         <s:f>G30*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I30" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11503,10 +11503,10 @@
       </s:c>
       <s:c r="J30" s="66">
         <s:f>I30+G30-H30</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K30" s="81" t="str">
-        <s:f>IF(F30&gt;B30,"Advance still growing",IF(F30&gt;0,"Paying it down",IF(G30&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F30&gt;B30,"Balance still growing",IF(F30&gt;0,"Working it down",IF(G30&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11525,7 +11525,7 @@
       </s:c>
       <s:c r="D31" s="76">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A31,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A31,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E31" s="76">
         <s:f>MIN(B31+C31,D31)</s:f>
@@ -11537,11 +11537,11 @@
       </s:c>
       <s:c r="G31" s="76">
         <s:f>MAX(0,D31-(B31+C31))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H31" s="76">
         <s:f>G31*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I31" s="67">
         <s:f>Inputs!$C$10</s:f>
@@ -11549,10 +11549,10 @@
       </s:c>
       <s:c r="J31" s="66">
         <s:f>I31+G31-H31</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K31" s="78" t="str">
-        <s:f>IF(F31&gt;B31,"Advance still growing",IF(F31&gt;0,"Paying it down",IF(G31&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F31&gt;B31,"Balance still growing",IF(F31&gt;0,"Working it down",IF(G31&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11571,7 +11571,7 @@
       </s:c>
       <s:c r="D32" s="79">
         <s:f>IF(SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A32,'Deal Log'!$H$9:$H$208,"Funded")&gt;0,SUMIFS('Deal Log'!$F$9:$F$208,'Deal Log'!$I$9:$I$208,A32,'Deal Log'!$H$9:$H$208,"Funded"),Inputs!$C$21)</s:f>
-        <s:v>4500.0</s:v>
+        <s:v>5250.0</s:v>
       </s:c>
       <s:c r="E32" s="79">
         <s:f>MIN(B32+C32,D32)</s:f>
@@ -11583,11 +11583,11 @@
       </s:c>
       <s:c r="G32" s="79">
         <s:f>MAX(0,D32-(B32+C32))</s:f>
-        <s:v>1500.0</s:v>
+        <s:v>2250.0</s:v>
       </s:c>
       <s:c r="H32" s="79">
         <s:f>G32*Inputs!$C$13</s:f>
-        <s:v>330.0</s:v>
+        <s:v>495.0</s:v>
       </s:c>
       <s:c r="I32" s="73">
         <s:f>Inputs!$C$10</s:f>
@@ -11595,10 +11595,10 @@
       </s:c>
       <s:c r="J32" s="66">
         <s:f>I32+G32-H32</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="K32" s="81" t="str">
-        <s:f>IF(F32&gt;B32,"Advance still growing",IF(F32&gt;0,"Paying it down",IF(G32&gt;0,"CLEARED - real income now","Cleared")))</s:f>
+        <s:f>IF(F32&gt;B32,"Balance still growing",IF(F32&gt;0,"Working it down",IF(G32&gt;0,"CLEARED - real income now","Cleared")))</s:f>
         <s:v>CLEARED - real income now</s:v>
       </s:c>
     </s:row>
@@ -11614,7 +11614,7 @@
       </s:c>
       <s:c r="D33" s="83">
         <s:f>SUM(D9:D32)</s:f>
-        <s:v>108000.0</s:v>
+        <s:v>126000.0</s:v>
       </s:c>
       <s:c r="E33" s="83">
         <s:f>SUM(E9:E32)</s:f>
@@ -11622,11 +11622,11 @@
       </s:c>
       <s:c r="G33" s="83">
         <s:f>SUM(G9:G32)</s:f>
-        <s:v>19500.0</s:v>
+        <s:v>37500.0</s:v>
       </s:c>
       <s:c r="H33" s="83">
         <s:f>SUM(H9:H32)</s:f>
-        <s:v>4290.0</s:v>
+        <s:v>8250.0</s:v>
       </s:c>
       <s:c r="I33" s="83">
         <s:f>SUM(I9:I32)</s:f>
@@ -11634,7 +11634,7 @@
       </s:c>
       <s:c r="J33" s="83">
         <s:f>SUM(J9:J32)</s:f>
-        <s:v>74325.84</s:v>
+        <s:v>88365.84</s:v>
       </s:c>
     </s:row>
   </s:sheetData>
@@ -11974,7 +11974,7 @@
       </s:c>
       <s:c r="D19" s="20" t="inlineStr">
         <s:is>
-          <s:t>Fixed at this until the advance clears - closing more loans does not change it.</s:t>
+          <s:t>Fixed at this until the balance is worked through - closing more loans does not change it yet.</s:t>
         </s:is>
       </s:c>
     </s:row>
@@ -12082,7 +12082,7 @@
       </s:c>
       <s:c r="D4" s="32">
         <s:f>AVERAGE(F9:F20)</s:f>
-        <s:v>-278.7994736842107</s:v>
+        <s:v>306.2005263157894</s:v>
       </s:c>
       <s:c r="E4" s="12" t="inlineStr">
         <s:is>
@@ -12091,7 +12091,7 @@
       </s:c>
       <s:c r="G4" s="31">
         <s:f>G32</s:f>
-        <s:v>6178.812631578945</s:v>
+        <s:v>20218.812631578945</s:v>
       </s:c>
     </s:row>
     <s:row r="8" ht="30" customHeight="1">
@@ -12414,7 +12414,7 @@
       </s:c>
       <s:c r="B16" s="73">
         <s:f>'Draw Payback'!J16</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>3633.16</s:v>
       </s:c>
       <s:c r="C16" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12430,11 +12430,11 @@
       </s:c>
       <s:c r="F16" s="86">
         <s:f>B16-E16</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>793.7005263157894</s:v>
       </s:c>
       <s:c r="G16" s="94">
         <s:f>G15+F16</s:f>
-        <s:v>-3010.395789473685</s:v>
+        <s:v>-1840.395789473685</s:v>
       </s:c>
       <s:c r="H16" s="73">
         <s:f>IF(MOD(7,3)=0,Inputs!$C$51,0)</s:f>
@@ -12442,7 +12442,7 @@
       </s:c>
       <s:c r="I16" s="81" t="str">
         <s:f>IF(F16&lt;0,"short - dipping into savings","")</s:f>
-        <s:v>short - dipping into savings</s:v>
+        <s:v/>
       </s:c>
     </s:row>
     <s:row r="17">
@@ -12452,7 +12452,7 @@
       </s:c>
       <s:c r="B17" s="67">
         <s:f>'Draw Payback'!J17</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C17" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12468,11 +12468,11 @@
       </s:c>
       <s:c r="F17" s="86">
         <s:f>B17-E17</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G17" s="77">
         <s:f>G16+F17</s:f>
-        <s:v>-3386.6952631578956</s:v>
+        <s:v>-461.6952631578956</s:v>
       </s:c>
       <s:c r="H17" s="67">
         <s:f>IF(MOD(8,3)=0,Inputs!$C$51,0)</s:f>
@@ -12480,7 +12480,7 @@
       </s:c>
       <s:c r="I17" s="78" t="str">
         <s:f>IF(F17&lt;0,"short - dipping into savings","")</s:f>
-        <s:v>short - dipping into savings</s:v>
+        <s:v/>
       </s:c>
     </s:row>
     <s:row r="18">
@@ -12490,7 +12490,7 @@
       </s:c>
       <s:c r="B18" s="73">
         <s:f>'Draw Payback'!J18</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C18" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12506,11 +12506,11 @@
       </s:c>
       <s:c r="F18" s="86">
         <s:f>B18-E18</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G18" s="94">
         <s:f>G17+F18</s:f>
-        <s:v>-3762.9947368421062</s:v>
+        <s:v>917.0052631578938</s:v>
       </s:c>
       <s:c r="H18" s="73">
         <s:f>IF(MOD(9,3)=0,Inputs!$C$51,0)</s:f>
@@ -12518,7 +12518,7 @@
       </s:c>
       <s:c r="I18" s="81" t="str">
         <s:f>IF(F18&lt;0,"short - dipping into savings","")</s:f>
-        <s:v>short - dipping into savings</s:v>
+        <s:v/>
       </s:c>
     </s:row>
     <s:row r="19">
@@ -12528,7 +12528,7 @@
       </s:c>
       <s:c r="B19" s="67">
         <s:f>'Draw Payback'!J19</s:f>
-        <s:v>2463.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C19" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12544,11 +12544,11 @@
       </s:c>
       <s:c r="F19" s="86">
         <s:f>B19-E19</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G19" s="77">
         <s:f>G18+F19</s:f>
-        <s:v>-4139.294210526317</s:v>
+        <s:v>2295.705789473683</s:v>
       </s:c>
       <s:c r="H19" s="67">
         <s:f>IF(MOD(10,3)=0,Inputs!$C$51,0)</s:f>
@@ -12556,7 +12556,7 @@
       </s:c>
       <s:c r="I19" s="78" t="str">
         <s:f>IF(F19&lt;0,"short - dipping into savings","")</s:f>
-        <s:v>short - dipping into savings</s:v>
+        <s:v/>
       </s:c>
     </s:row>
     <s:row r="20">
@@ -12566,7 +12566,7 @@
       </s:c>
       <s:c r="B20" s="73">
         <s:f>'Draw Payback'!J20</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C20" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12582,11 +12582,11 @@
       </s:c>
       <s:c r="F20" s="86">
         <s:f>B20-E20</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G20" s="94">
         <s:f>G19+F20</s:f>
-        <s:v>-3345.593684210528</s:v>
+        <s:v>3674.4063157894725</s:v>
       </s:c>
       <s:c r="H20" s="73">
         <s:f>IF(MOD(11,3)=0,Inputs!$C$51,0)</s:f>
@@ -12604,7 +12604,7 @@
       </s:c>
       <s:c r="B21" s="67">
         <s:f>'Draw Payback'!J21</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C21" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12620,11 +12620,11 @@
       </s:c>
       <s:c r="F21" s="86">
         <s:f>B21-E21</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G21" s="77">
         <s:f>G20+F21</s:f>
-        <s:v>-2551.8931578947386</s:v>
+        <s:v>5053.106842105262</s:v>
       </s:c>
       <s:c r="H21" s="67">
         <s:f>IF(MOD(12,3)=0,Inputs!$C$51,0)</s:f>
@@ -12642,7 +12642,7 @@
       </s:c>
       <s:c r="B22" s="73">
         <s:f>'Draw Payback'!J22</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C22" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12658,11 +12658,11 @@
       </s:c>
       <s:c r="F22" s="86">
         <s:f>B22-E22</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G22" s="94">
         <s:f>G21+F22</s:f>
-        <s:v>-1758.1926315789492</s:v>
+        <s:v>6431.807368421052</s:v>
       </s:c>
       <s:c r="H22" s="73">
         <s:f>IF(MOD(13,3)=0,Inputs!$C$51,0)</s:f>
@@ -12680,7 +12680,7 @@
       </s:c>
       <s:c r="B23" s="67">
         <s:f>'Draw Payback'!J23</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C23" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12696,11 +12696,11 @@
       </s:c>
       <s:c r="F23" s="86">
         <s:f>B23-E23</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G23" s="77">
         <s:f>G22+F23</s:f>
-        <s:v>-964.4921052631598</s:v>
+        <s:v>7810.507894736842</s:v>
       </s:c>
       <s:c r="H23" s="67">
         <s:f>IF(MOD(14,3)=0,Inputs!$C$51,0)</s:f>
@@ -12718,7 +12718,7 @@
       </s:c>
       <s:c r="B24" s="73">
         <s:f>'Draw Payback'!J24</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C24" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12734,11 +12734,11 @@
       </s:c>
       <s:c r="F24" s="86">
         <s:f>B24-E24</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G24" s="94">
         <s:f>G23+F24</s:f>
-        <s:v>-170.79157894737045</s:v>
+        <s:v>9189.208421052632</s:v>
       </s:c>
       <s:c r="H24" s="73">
         <s:f>IF(MOD(15,3)=0,Inputs!$C$51,0)</s:f>
@@ -12756,7 +12756,7 @@
       </s:c>
       <s:c r="B25" s="67">
         <s:f>'Draw Payback'!J25</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C25" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12772,11 +12772,11 @@
       </s:c>
       <s:c r="F25" s="86">
         <s:f>B25-E25</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G25" s="77">
         <s:f>G24+F25</s:f>
-        <s:v>622.9089473684189</s:v>
+        <s:v>10567.908947368422</s:v>
       </s:c>
       <s:c r="H25" s="67">
         <s:f>IF(MOD(16,3)=0,Inputs!$C$51,0)</s:f>
@@ -12794,7 +12794,7 @@
       </s:c>
       <s:c r="B26" s="73">
         <s:f>'Draw Payback'!J26</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C26" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12810,11 +12810,11 @@
       </s:c>
       <s:c r="F26" s="86">
         <s:f>B26-E26</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G26" s="94">
         <s:f>G25+F26</s:f>
-        <s:v>1416.6094736842083</s:v>
+        <s:v>11946.609473684211</s:v>
       </s:c>
       <s:c r="H26" s="73">
         <s:f>IF(MOD(17,3)=0,Inputs!$C$51,0)</s:f>
@@ -12832,7 +12832,7 @@
       </s:c>
       <s:c r="B27" s="67">
         <s:f>'Draw Payback'!J27</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C27" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12848,11 +12848,11 @@
       </s:c>
       <s:c r="F27" s="86">
         <s:f>B27-E27</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G27" s="77">
         <s:f>G26+F27</s:f>
-        <s:v>2210.3099999999977</s:v>
+        <s:v>13325.310000000001</s:v>
       </s:c>
       <s:c r="H27" s="67">
         <s:f>IF(MOD(18,3)=0,Inputs!$C$51,0)</s:f>
@@ -12870,7 +12870,7 @@
       </s:c>
       <s:c r="B28" s="73">
         <s:f>'Draw Payback'!J28</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C28" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12886,11 +12886,11 @@
       </s:c>
       <s:c r="F28" s="86">
         <s:f>B28-E28</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G28" s="94">
         <s:f>G27+F28</s:f>
-        <s:v>3004.010526315787</s:v>
+        <s:v>14704.010526315791</s:v>
       </s:c>
       <s:c r="H28" s="73">
         <s:f>IF(MOD(19,3)=0,Inputs!$C$51,0)</s:f>
@@ -12908,7 +12908,7 @@
       </s:c>
       <s:c r="B29" s="67">
         <s:f>'Draw Payback'!J29</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C29" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -12924,11 +12924,11 @@
       </s:c>
       <s:c r="F29" s="86">
         <s:f>B29-E29</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G29" s="77">
         <s:f>G28+F29</s:f>
-        <s:v>3797.7110526315764</s:v>
+        <s:v>16082.711052631581</s:v>
       </s:c>
       <s:c r="H29" s="67">
         <s:f>IF(MOD(20,3)=0,Inputs!$C$51,0)</s:f>
@@ -12946,7 +12946,7 @@
       </s:c>
       <s:c r="B30" s="73">
         <s:f>'Draw Payback'!J30</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C30" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -12962,11 +12962,11 @@
       </s:c>
       <s:c r="F30" s="86">
         <s:f>B30-E30</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G30" s="94">
         <s:f>G29+F30</s:f>
-        <s:v>4591.411578947365</s:v>
+        <s:v>17461.41157894737</s:v>
       </s:c>
       <s:c r="H30" s="73">
         <s:f>IF(MOD(21,3)=0,Inputs!$C$51,0)</s:f>
@@ -12984,7 +12984,7 @@
       </s:c>
       <s:c r="B31" s="67">
         <s:f>'Draw Payback'!J31</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C31" s="67">
         <s:f>Budget!$B$15</s:f>
@@ -13000,11 +13000,11 @@
       </s:c>
       <s:c r="F31" s="86">
         <s:f>B31-E31</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G31" s="77">
         <s:f>G30+F31</s:f>
-        <s:v>5385.112105263155</s:v>
+        <s:v>18840.112105263157</s:v>
       </s:c>
       <s:c r="H31" s="67">
         <s:f>IF(MOD(22,3)=0,Inputs!$C$51,0)</s:f>
@@ -13022,7 +13022,7 @@
       </s:c>
       <s:c r="B32" s="73">
         <s:f>'Draw Payback'!J32</s:f>
-        <s:v>3633.16</s:v>
+        <s:v>4218.16</s:v>
       </s:c>
       <s:c r="C32" s="73">
         <s:f>Budget!$B$15</s:f>
@@ -13038,11 +13038,11 @@
       </s:c>
       <s:c r="F32" s="86">
         <s:f>B32-E32</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="G32" s="94">
         <s:f>G31+F32</s:f>
-        <s:v>6178.812631578945</s:v>
+        <s:v>20218.812631578945</s:v>
       </s:c>
       <s:c r="H32" s="73">
         <s:f>IF(MOD(23,3)=0,Inputs!$C$51,0)</s:f>
@@ -13061,7 +13061,7 @@
       </s:c>
       <s:c r="B33" s="83">
         <s:f>SUM(B9:B32)</s:f>
-        <s:v>74325.84</s:v>
+        <s:v>88365.84</s:v>
       </s:c>
       <s:c r="C33" s="83">
         <s:f>SUM(C9:C32)</s:f>
@@ -13077,7 +13077,7 @@
       </s:c>
       <s:c r="F33" s="83">
         <s:f>SUM(F9:F32)</s:f>
-        <s:v>6178.812631578945</s:v>
+        <s:v>20218.812631578945</s:v>
       </s:c>
     </s:row>
   </s:sheetData>
@@ -13521,11 +13521,11 @@
       </s:c>
       <s:c r="B16" s="73">
         <s:f>'Cash Flow'!F16</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>793.7005263157894</s:v>
       </s:c>
       <s:c r="C16" s="94">
         <s:f>C15+IF(B16&lt;0,B16,MIN(B16,Inputs!$C$45-C15))</s:f>
-        <s:v>-2614.995789473685</s:v>
+        <s:v>-1444.995789473685</s:v>
       </s:c>
       <s:c r="D16" s="94">
         <s:f>D15*(1+Inputs!$C$47/12)+IF(D15&lt;Inputs!$C$60*Budget!B17,MAX(0,B16-(C16-C15)),MAX(0,B16-(C16-C15))*0.30)-'Cash Flow'!H16</s:f>
@@ -13549,11 +13549,11 @@
       </s:c>
       <s:c r="I16" s="66">
         <s:f>C16+D16+E16+F16+G16</s:f>
-        <s:v>12691.309053442921</s:v>
+        <s:v>13861.309053442921</s:v>
       </s:c>
       <s:c r="J16" s="86">
         <s:f>I16-H16</s:f>
-        <s:v>-9791.654077521096</s:v>
+        <s:v>-8621.654077521096</s:v>
       </s:c>
     </s:row>
     <s:row r="17">
@@ -13563,11 +13563,11 @@
       </s:c>
       <s:c r="B17" s="67">
         <s:f>'Cash Flow'!F17</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C17" s="77">
         <s:f>C16+IF(B17&lt;0,B17,MIN(B17,Inputs!$C$45-C16))</s:f>
-        <s:v>-2991.2952631578955</s:v>
+        <s:v>-66.29526315789553</s:v>
       </s:c>
       <s:c r="D17" s="77">
         <s:f>D16*(1+Inputs!$C$47/12)+IF(D16&lt;Inputs!$C$60*Budget!B17,MAX(0,B17-(C17-C16)),MAX(0,B17-(C17-C16))*0.30)-'Cash Flow'!H17</s:f>
@@ -13591,11 +13591,11 @@
       </s:c>
       <s:c r="I17" s="66">
         <s:f>C17+D17+E17+F17+G17</s:f>
-        <s:v>12363.296754653758</s:v>
+        <s:v>15288.296754653758</s:v>
       </s:c>
       <s:c r="J17" s="86">
         <s:f>I17-H17</s:f>
-        <s:v>-9784.307537852696</s:v>
+        <s:v>-6859.3075378526955</s:v>
       </s:c>
     </s:row>
     <s:row r="18">
@@ -13605,11 +13605,11 @@
       </s:c>
       <s:c r="B18" s="73">
         <s:f>'Cash Flow'!F18</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C18" s="94">
         <s:f>C17+IF(B18&lt;0,B18,MIN(B18,Inputs!$C$45-C17))</s:f>
-        <s:v>-3367.594736842106</s:v>
+        <s:v>1312.4052631578938</s:v>
       </s:c>
       <s:c r="D18" s="94">
         <s:f>D17*(1+Inputs!$C$47/12)+IF(D17&lt;Inputs!$C$60*Budget!B17,MAX(0,B18-(C18-C17)),MAX(0,B18-(C18-C17))*0.30)-'Cash Flow'!H18</s:f>
@@ -13633,11 +13633,11 @@
       </s:c>
       <s:c r="I18" s="66">
         <s:f>C18+D18+E18+F18+G18</s:f>
-        <s:v>12035.437013387012</s:v>
+        <s:v>16715.43701338701</s:v>
       </s:c>
       <s:c r="J18" s="86">
         <s:f>I18-H18</s:f>
-        <s:v>-9774.715242578504</s:v>
+        <s:v>-5094.715242578506</s:v>
       </s:c>
     </s:row>
     <s:row r="19">
@@ -13647,15 +13647,15 @@
       </s:c>
       <s:c r="B19" s="67">
         <s:f>'Cash Flow'!F19</s:f>
-        <s:v>-376.2994736842106</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C19" s="77">
         <s:f>C18+IF(B19&lt;0,B19,MIN(B19,Inputs!$C$45-C18))</s:f>
-        <s:v>-3743.894210526317</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D19" s="77">
         <s:f>D18*(1+Inputs!$C$47/12)+IF(D18&lt;Inputs!$C$60*Budget!B17,MAX(0,B19-(C19-C18)),MAX(0,B19-(C19-C18))*0.30)-'Cash Flow'!H19</s:f>
-        <s:v>3619.3699322869197</s:v>
+        <s:v>4310.475721760603</s:v>
       </s:c>
       <s:c r="E19" s="77">
         <s:f>E18*(1+Inputs!$C$49/12)+'Cash Flow'!H19</s:f>
@@ -13675,11 +13675,11 @@
       </s:c>
       <s:c r="I19" s="66">
         <s:f>C19+D19+E19+F19+G19</s:f>
-        <s:v>11707.404270692929</s:v>
+        <s:v>18142.40427069293</s:v>
       </s:c>
       <s:c r="J19" s="86">
         <s:f>I19-H19</s:f>
-        <s:v>-9763.189685603575</s:v>
+        <s:v>-3328.1896856035746</s:v>
       </s:c>
     </s:row>
     <s:row r="20">
@@ -13689,15 +13689,15 @@
       </s:c>
       <s:c r="B20" s="73">
         <s:f>'Cash Flow'!F20</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C20" s="94">
         <s:f>C19+IF(B20&lt;0,B20,MIN(B20,Inputs!$C$45-C19))</s:f>
-        <s:v>-2950.1936842105274</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D20" s="94">
         <s:f>D19*(1+Inputs!$C$47/12)+IF(D19&lt;Inputs!$C$60*Budget!B17,MAX(0,B20-(C20-C19)),MAX(0,B20-(C20-C19))*0.30)-'Cash Flow'!H20</s:f>
-        <s:v>3631.4344987278764</s:v>
+        <s:v>5703.544500482261</s:v>
       </s:c>
       <s:c r="E20" s="94">
         <s:f>E19*(1+Inputs!$C$49/12)+'Cash Flow'!H20</s:f>
@@ -13717,11 +13717,11 @@
       </s:c>
       <s:c r="I20" s="66">
         <s:f>C20+D20+E20+F20+G20</s:f>
-        <s:v>12549.522963916268</s:v>
+        <s:v>19571.82664988118</s:v>
       </s:c>
       <s:c r="J20" s="86">
         <s:f>I20-H20</s:f>
-        <s:v>-8579.393282990786</s:v>
+        <s:v>-1557.0895970258753</s:v>
       </s:c>
     </s:row>
     <s:row r="21">
@@ -13731,15 +13731,15 @@
       </s:c>
       <s:c r="B21" s="67">
         <s:f>'Cash Flow'!F21</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C21" s="77">
         <s:f>C20+IF(B21&lt;0,B21,MIN(B21,Inputs!$C$45-C20))</s:f>
-        <s:v>-2156.493157894738</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D21" s="77">
         <s:f>D20*(1+Inputs!$C$47/12)+IF(D20&lt;Inputs!$C$60*Budget!B17,MAX(0,B21-(C21-C20)),MAX(0,B21-(C21-C20))*0.30)-'Cash Flow'!H21</s:f>
-        <s:v>2393.539280390303</s:v>
+        <s:v>5851.256841799659</s:v>
       </s:c>
       <s:c r="E21" s="77">
         <s:f>E20*(1+Inputs!$C$49/12)+'Cash Flow'!H21</s:f>
@@ -13759,11 +13759,11 @@
       </s:c>
       <s:c r="I21" s="66">
         <s:f>C21+D21+E21+F21+G21</s:f>
-        <s:v>13391.793568798514</s:v>
+        <s:v>21006.00428810261</s:v>
       </s:c>
       <s:c r="J21" s="86">
         <s:f>I21-H21</s:f>
-        <s:v>-7393.312330349652</s:v>
+        <s:v>220.89838895444336</s:v>
       </s:c>
     </s:row>
     <s:row r="22">
@@ -13773,15 +13773,15 @@
       </s:c>
       <s:c r="B22" s="73">
         <s:f>'Cash Flow'!F22</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C22" s="94">
         <s:f>C21+IF(B22&lt;0,B22,MIN(B22,Inputs!$C$45-C21))</s:f>
-        <s:v>-1362.7926315789487</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D22" s="94">
         <s:f>D21*(1+Inputs!$C$47/12)+IF(D21&lt;Inputs!$C$60*Budget!B17,MAX(0,B22-(C22-C21)),MAX(0,B22-(C22-C21))*0.30)-'Cash Flow'!H22</s:f>
-        <s:v>2401.5177446582707</s:v>
+        <s:v>7249.461557588114</s:v>
       </s:c>
       <s:c r="E22" s="94">
         <s:f>E21*(1+Inputs!$C$49/12)+'Cash Flow'!H22</s:f>
@@ -13801,11 +13801,11 @@
       </s:c>
       <s:c r="I22" s="66">
         <s:f>C22+D22+E22+F22+G22</s:f>
-        <s:v>14233.890520911038</s:v>
+        <s:v>22444.62696541983</s:v>
       </s:c>
       <s:c r="J22" s="86">
         <s:f>I22-H22</s:f>
-        <s:v>-6205.259080890977</s:v>
+        <s:v>2005.4773636178143</s:v>
       </s:c>
     </s:row>
     <s:row r="23">
@@ -13815,15 +13815,15 @@
       </s:c>
       <s:c r="B23" s="67">
         <s:f>'Cash Flow'!F23</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C23" s="77">
         <s:f>C22+IF(B23&lt;0,B23,MIN(B23,Inputs!$C$45-C22))</s:f>
-        <s:v>-569.0921052631593</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D23" s="77">
         <s:f>D22*(1+Inputs!$C$47/12)+IF(D22&lt;Inputs!$C$60*Budget!B17,MAX(0,B23-(C23-C22)),MAX(0,B23-(C23-C22))*0.30)-'Cash Flow'!H23</s:f>
-        <s:v>2409.522803807132</s:v>
+        <s:v>8652.326955762532</s:v>
       </s:c>
       <s:c r="E23" s="77">
         <s:f>E22*(1+Inputs!$C$49/12)+'Cash Flow'!H23</s:f>
@@ -13843,11 +13843,11 @@
       </s:c>
       <s:c r="I23" s="66">
         <s:f>C23+D23+E23+F23+G23</s:f>
-        <s:v>15076.13825209125</s:v>
+        <s:v>23888.034509309808</s:v>
       </s:c>
       <s:c r="J23" s="86">
         <s:f>I23-H23</s:f>
-        <s:v>-5014.895708475347</s:v>
+        <s:v>3797.00054874321</s:v>
       </s:c>
     </s:row>
     <s:row r="24">
@@ -13857,15 +13857,15 @@
       </s:c>
       <s:c r="B24" s="73">
         <s:f>'Cash Flow'!F24</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C24" s="94">
         <s:f>C23+IF(B24&lt;0,B24,MIN(B24,Inputs!$C$45-C23))</s:f>
-        <s:v>224.6084210526301</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D24" s="94">
         <s:f>D23*(1+Inputs!$C$47/12)+IF(D23&lt;Inputs!$C$60*Budget!B17,MAX(0,B24-(C24-C23)),MAX(0,B24-(C24-C23))*0.30)-'Cash Flow'!H24</s:f>
-        <s:v>1167.554546486489</s:v>
+        <s:v>8809.868571930863</s:v>
       </s:c>
       <s:c r="E24" s="94">
         <s:f>E23*(1+Inputs!$C$49/12)+'Cash Flow'!H24</s:f>
@@ -13885,11 +13885,11 @@
       </s:c>
       <s:c r="I24" s="66">
         <s:f>C24+D24+E24+F24+G24</s:f>
-        <s:v>15918.537232544671</s:v>
+        <s:v>25336.242836936413</s:v>
       </s:c>
       <s:c r="J24" s="86">
         <s:f>I24-H24</s:f>
-        <s:v>-3822.208264992465</s:v>
+        <s:v>5595.497339399277</s:v>
       </s:c>
     </s:row>
     <s:row r="25">
@@ -13899,15 +13899,15 @@
       </s:c>
       <s:c r="B25" s="67">
         <s:f>'Cash Flow'!F25</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C25" s="77">
         <s:f>C24+IF(B25&lt;0,B25,MIN(B25,Inputs!$C$45-C24))</s:f>
-        <s:v>1018.3089473684195</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D25" s="77">
         <s:f>D24*(1+Inputs!$C$47/12)+IF(D24&lt;Inputs!$C$60*Budget!B17,MAX(0,B25-(C25-C24)),MAX(0,B25-(C25-C24))*0.30)-'Cash Flow'!H25</s:f>
-        <s:v>1171.4463949747774</s:v>
+        <s:v>10217.935326819757</s:v>
       </s:c>
       <s:c r="E25" s="77">
         <s:f>E24*(1+Inputs!$C$49/12)+'Cash Flow'!H25</s:f>
@@ -13927,11 +13927,11 @@
       </s:c>
       <s:c r="I25" s="66">
         <s:f>C25+D25+E25+F25+G25</s:f>
-        <s:v>16760.76189227798</s:v>
+        <s:v>26788.94187675454</s:v>
       </s:c>
       <s:c r="J25" s="86">
         <s:f>I25-H25</s:f>
-        <s:v>-2627.508758406286</s:v>
+        <s:v>7400.671226070273</s:v>
       </s:c>
     </s:row>
     <s:row r="26">
@@ -13941,15 +13941,15 @@
       </s:c>
       <s:c r="B26" s="73">
         <s:f>'Cash Flow'!F26</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C26" s="94">
         <s:f>C25+IF(B26&lt;0,B26,MIN(B26,Inputs!$C$45-C25))</s:f>
-        <s:v>1812.0094736842088</s:v>
+        <s:v>2000.0</s:v>
       </s:c>
       <s:c r="D26" s="94">
         <s:f>D25*(1+Inputs!$C$47/12)+IF(D25&lt;Inputs!$C$60*Budget!B17,MAX(0,B26-(C26-C25)),MAX(0,B26-(C26-C25))*0.30)-'Cash Flow'!H26</s:f>
-        <s:v>1175.35121629136</s:v>
+        <s:v>11630.695637558281</s:v>
       </s:c>
       <s:c r="E26" s="94">
         <s:f>E25*(1+Inputs!$C$49/12)+'Cash Flow'!H26</s:f>
@@ -13969,11 +13969,11 @@
       </s:c>
       <s:c r="I26" s="66">
         <s:f>C26+D26+E26+F26+G26</s:f>
-        <s:v>17603.136657535026</s:v>
+        <s:v>28246.47160511774</s:v>
       </s:c>
       <s:c r="J26" s="86">
         <s:f>I26-H26</s:f>
-        <s:v>-1430.4591157939285</s:v>
+        <s:v>9212.875831788784</s:v>
       </s:c>
     </s:row>
     <s:row r="27">
@@ -13983,7 +13983,7 @@
       </s:c>
       <s:c r="B27" s="67">
         <s:f>'Cash Flow'!F27</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C27" s="77">
         <s:f>C26+IF(B27&lt;0,B27,MIN(B27,Inputs!$C$45-C26))</s:f>
@@ -13991,7 +13991,7 @@
       </s:c>
       <s:c r="D27" s="77">
         <s:f>D26*(1+Inputs!$C$47/12)+IF(D26&lt;Inputs!$C$60*Budget!B17,MAX(0,B27-(C27-C26)),MAX(0,B27-(C27-C26))*0.30)-'Cash Flow'!H27</s:f>
-        <s:v>534.9790536789963</s:v>
+        <s:v>11798.165149332599</s:v>
       </s:c>
       <s:c r="E27" s="77">
         <s:f>E26*(1+Inputs!$C$49/12)+'Cash Flow'!H27</s:f>
@@ -14011,11 +14011,11 @@
       </s:c>
       <s:c r="I27" s="66">
         <s:f>C27+D27+E27+F27+G27</s:f>
-        <s:v>18445.66199289878</s:v>
+        <s:v>29708.848088552382</s:v>
       </s:c>
       <s:c r="J27" s="86">
         <s:f>I27-H27</s:f>
-        <s:v>-231.0451407153705</s:v>
+        <s:v>11032.140954938233</s:v>
       </s:c>
     </s:row>
     <s:row r="28">
@@ -14025,7 +14025,7 @@
       </s:c>
       <s:c r="B28" s="73">
         <s:f>'Cash Flow'!F28</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C28" s="94">
         <s:f>C27+IF(B28&lt;0,B28,MIN(B28,Inputs!$C$45-C27))</s:f>
@@ -14033,7 +14033,7 @@
       </s:c>
       <s:c r="D28" s="94">
         <s:f>D27*(1+Inputs!$C$47/12)+IF(D27&lt;Inputs!$C$60*Budget!B17,MAX(0,B28-(C28-C27)),MAX(0,B28-(C28-C27))*0.30)-'Cash Flow'!H28</s:f>
-        <s:v>1330.462843507049</s:v>
+        <s:v>13216.19289281283</s:v>
       </s:c>
       <s:c r="E28" s="94">
         <s:f>E27*(1+Inputs!$C$49/12)+'Cash Flow'!H28</s:f>
@@ -14053,11 +14053,11 @@
       </s:c>
       <s:c r="I28" s="66">
         <s:f>C28+D28+E28+F28+G28</s:f>
-        <s:v>19290.031356057585</s:v>
+        <s:v>31175.761405363366</s:v>
       </s:c>
       <s:c r="J28" s="86">
         <s:f>I28-H28</s:f>
-        <s:v>972.4404420844585</s:v>
+        <s:v>12858.17049139024</s:v>
       </s:c>
     </s:row>
     <s:row r="29">
@@ -14067,7 +14067,7 @@
       </s:c>
       <s:c r="B29" s="67">
         <s:f>'Cash Flow'!F29</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C29" s="77">
         <s:f>C28+IF(B29&lt;0,B29,MIN(B29,Inputs!$C$45-C28))</s:f>
@@ -14075,7 +14075,7 @@
       </s:c>
       <s:c r="D29" s="77">
         <s:f>D28*(1+Inputs!$C$47/12)+IF(D28&lt;Inputs!$C$60*Budget!B17,MAX(0,B29-(C29-C28)),MAX(0,B29-(C29-C28))*0.30)-'Cash Flow'!H29</s:f>
-        <s:v>2128.5982459678617</s:v>
+        <s:v>14638.947395437997</s:v>
       </s:c>
       <s:c r="E29" s="77">
         <s:f>E28*(1+Inputs!$C$49/12)+'Cash Flow'!H29</s:f>
@@ -14095,11 +14095,11 @@
       </s:c>
       <s:c r="I29" s="66">
         <s:f>C29+D29+E29+F29+G29</s:f>
-        <s:v>20137.20253277321</s:v>
+        <s:v>32647.551682243346</s:v>
       </s:c>
       <s:c r="J29" s="86">
         <s:f>I29-H29</s:f>
-        <s:v>2180.969322178702</s:v>
+        <s:v>14691.318471648836</s:v>
       </s:c>
     </s:row>
     <s:row r="30">
@@ -14109,7 +14109,7 @@
       </s:c>
       <s:c r="B30" s="73">
         <s:f>'Cash Flow'!F30</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C30" s="94">
         <s:f>C29+IF(B30&lt;0,B30,MIN(B30,Inputs!$C$45-C29))</s:f>
@@ -14117,7 +14117,7 @@
       </s:c>
       <s:c r="D30" s="94">
         <s:f>D29*(1+Inputs!$C$47/12)+IF(D29&lt;Inputs!$C$60*Budget!B17,MAX(0,B30-(C30-C29)),MAX(0,B30-(C30-C29))*0.30)-'Cash Flow'!H30</s:f>
-        <s:v>1679.3940997702107</s:v>
+        <s:v>14816.444413071915</s:v>
       </s:c>
       <s:c r="E30" s="94">
         <s:f>E29*(1+Inputs!$C$49/12)+'Cash Flow'!H30</s:f>
@@ -14137,11 +14137,11 @@
       </s:c>
       <s:c r="I30" s="66">
         <s:f>C30+D30+E30+F30+G30</s:f>
-        <s:v>20987.18482324677</s:v>
+        <s:v>34124.23513654847</s:v>
       </s:c>
       <s:c r="J30" s="86">
         <s:f>I30-H30</s:f>
-        <s:v>3394.564790362798</s:v>
+        <s:v>16531.6151036645</s:v>
       </s:c>
     </s:row>
     <s:row r="31">
@@ -14151,7 +14151,7 @@
       </s:c>
       <s:c r="B31" s="67">
         <s:f>'Cash Flow'!F31</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C31" s="77">
         <s:f>C30+IF(B31&lt;0,B31,MIN(B31,Inputs!$C$45-C30))</s:f>
@@ -14159,7 +14159,7 @@
       </s:c>
       <s:c r="D31" s="77">
         <s:f>D30*(1+Inputs!$C$47/12)+IF(D30&lt;Inputs!$C$60*Budget!B17,MAX(0,B31-(C31-C30)),MAX(0,B31-(C31-C30))*0.30)-'Cash Flow'!H31</s:f>
-        <s:v>2478.6926064185673</s:v>
+        <s:v>16244.533087431279</s:v>
       </s:c>
       <s:c r="E31" s="77">
         <s:f>E30*(1+Inputs!$C$49/12)+'Cash Flow'!H31</s:f>
@@ -14179,11 +14179,11 @@
       </s:c>
       <s:c r="I31" s="66">
         <s:f>C31+D31+E31+F31+G31</s:f>
-        <s:v>21839.66151689301</s:v>
+        <s:v>35605.501997905725</s:v>
       </s:c>
       <s:c r="J31" s="86">
         <s:f>I31-H31</s:f>
-        <s:v>4612.924213970451</s:v>
+        <s:v>18378.764694983165</s:v>
       </s:c>
     </s:row>
     <s:row r="32">
@@ -14193,7 +14193,7 @@
       </s:c>
       <s:c r="B32" s="73">
         <s:f>'Cash Flow'!F32</s:f>
-        <s:v>793.7005263157894</s:v>
+        <s:v>1378.7005263157894</s:v>
       </s:c>
       <s:c r="C32" s="94">
         <s:f>C31+IF(B32&lt;0,B32,MIN(B32,Inputs!$C$45-C31))</s:f>
@@ -14201,7 +14201,7 @@
       </s:c>
       <s:c r="D32" s="94">
         <s:f>D31*(1+Inputs!$C$47/12)+IF(D31&lt;Inputs!$C$60*Budget!B17,MAX(0,B32-(C32-C31)),MAX(0,B32-(C32-C31))*0.30)-'Cash Flow'!H32</s:f>
-        <s:v>3280.655441422419</s:v>
+        <s:v>17677.38205737184</s:v>
       </s:c>
       <s:c r="E32" s="94">
         <s:f>E31*(1+Inputs!$C$49/12)+'Cash Flow'!H32</s:f>
@@ -14221,11 +14221,11 @@
       </s:c>
       <s:c r="I32" s="66">
         <s:f>C32+D32+E32+F32+G32</s:f>
-        <s:v>22694.965928874295</s:v>
+        <s:v>37091.692544823716</s:v>
       </s:c>
       <s:c r="J32" s="86">
         <s:f>I32-H32</s:f>
-        <s:v>5836.395073952659</s:v>
+        <s:v>20233.12168990208</s:v>
       </s:c>
     </s:row>
   </s:sheetData>

</xml_diff>